<commit_message>
#14 Client and JLCPCB BOM update Peripherals remaining.
</commit_message>
<xml_diff>
--- a/Design Files/DC-Motor-Driver/BOM/Client_BOM-v2.0.xlsx
+++ b/Design Files/DC-Motor-Driver/BOM/Client_BOM-v2.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\manarharake-motordriver\Design Files\DC-Motor-Driver\Project Outputs for DC-Motor-Driver-v1.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\manarharake-motordriver\Design Files\DC-Motor-Driver\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="343">
   <si>
     <t>#</t>
   </si>
@@ -63,6 +63,9 @@
     <t>Resistor</t>
   </si>
   <si>
+    <t>Resistors</t>
+  </si>
+  <si>
     <t>Switch</t>
   </si>
   <si>
@@ -969,9 +972,6 @@
     <t>1uH</t>
   </si>
   <si>
-    <t>Orange</t>
-  </si>
-  <si>
     <t>100K</t>
   </si>
   <si>
@@ -1032,23 +1032,29 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>Value</t>
+  </si>
+  <si>
     <t>LED</t>
   </si>
   <si>
-    <t>Value</t>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Do Not Place</t>
   </si>
   <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>-</t>
+    <t>XL-2012UOC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1087,6 +1093,14 @@
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1207,7 +1221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1246,6 +1260,18 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1544,9 +1570,9 @@
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1571,28 +1597,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>336</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1605,22 +1631,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J3" s="7">
         <v>4</v>
@@ -1637,22 +1663,22 @@
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J4" s="9">
         <v>20</v>
@@ -1669,22 +1695,22 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J5" s="7">
         <v>9</v>
@@ -1697,26 +1723,26 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J6" s="9">
         <v>27</v>
@@ -1733,22 +1759,22 @@
         <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J7" s="7">
         <v>5</v>
@@ -1765,22 +1791,22 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J8" s="9">
         <v>4</v>
@@ -1797,22 +1823,22 @@
         <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1829,22 +1855,22 @@
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J10" s="9">
         <v>3</v>
@@ -1861,22 +1887,22 @@
         <v>2</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J11" s="7">
         <v>6</v>
@@ -1889,26 +1915,26 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J12" s="9">
         <v>6</v>
@@ -1925,22 +1951,22 @@
         <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1953,26 +1979,26 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1985,26 +2011,26 @@
         <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -2017,26 +2043,26 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
@@ -2053,22 +2079,22 @@
         <v>2</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -2085,22 +2111,22 @@
         <v>2</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -2117,22 +2143,22 @@
         <v>3</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J19" s="7">
         <v>3</v>
@@ -2149,22 +2175,22 @@
         <v>3</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>270</v>
-      </c>
-      <c r="I20" s="10" t="s">
-        <v>340</v>
+        <v>271</v>
+      </c>
+      <c r="I20" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="J20" s="9">
         <v>2</v>
@@ -2181,22 +2207,22 @@
         <v>3</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -2213,22 +2239,22 @@
         <v>3</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>269</v>
-      </c>
-      <c r="I22" s="10" t="s">
-        <v>340</v>
+        <v>270</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -2245,22 +2271,22 @@
         <v>3</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2277,22 +2303,22 @@
         <v>4</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="I24" s="10" t="s">
-        <v>340</v>
+        <v>274</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2309,22 +2335,22 @@
         <v>5</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J25" s="7">
         <v>2</v>
@@ -2337,26 +2363,24 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C26" s="13" t="s">
-        <v>7</v>
-      </c>
+      <c r="C26" s="13"/>
       <c r="D26" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>274</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>340</v>
+        <v>275</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="J26" s="9">
         <v>6</v>
@@ -2373,22 +2397,22 @@
         <v>6</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2405,22 +2429,22 @@
         <v>7</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>276</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>340</v>
+        <v>277</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2437,22 +2461,22 @@
         <v>8</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2469,22 +2493,22 @@
         <v>9</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>340</v>
+        <v>278</v>
+      </c>
+      <c r="I30" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="J30" s="9">
         <v>2</v>
@@ -2501,22 +2525,22 @@
         <v>7</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2533,22 +2557,22 @@
         <v>10</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2565,22 +2589,22 @@
         <v>10</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2597,22 +2621,22 @@
         <v>10</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2626,23 +2650,25 @@
         <v>33</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="G35" s="8"/>
+        <v>180</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>342</v>
+      </c>
       <c r="H35" s="7" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>316</v>
+        <v>339</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2659,22 +2685,22 @@
         <v>11</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="I36" s="10" t="s">
-        <v>340</v>
+        <v>283</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2691,22 +2717,22 @@
         <v>11</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J37" s="7">
         <v>2</v>
@@ -2723,22 +2749,22 @@
         <v>12</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>284</v>
-      </c>
-      <c r="I38" s="10" t="s">
-        <v>340</v>
+        <v>285</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>339</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
@@ -2755,19 +2781,19 @@
         <v>13</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>317</v>
@@ -2787,19 +2813,19 @@
         <v>13</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I40" s="10" t="s">
         <v>318</v>
@@ -2819,19 +2845,19 @@
         <v>13</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>319</v>
@@ -2851,19 +2877,19 @@
         <v>13</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="I42" s="10" t="s">
         <v>320</v>
@@ -2883,19 +2909,19 @@
         <v>13</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>321</v>
@@ -2914,28 +2940,30 @@
       <c r="C44" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D44" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="G44" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="H44" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="I44" s="10" t="s">
+      <c r="D44" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="E44" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="F44" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="G44" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="H44" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="I44" s="18" t="s">
         <v>322</v>
       </c>
-      <c r="J44" s="9">
-        <v>1</v>
-      </c>
-      <c r="K44" s="9"/>
+      <c r="J44" s="17">
+        <v>1</v>
+      </c>
+      <c r="K44" s="15" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="45" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
@@ -2947,19 +2975,19 @@
         <v>13</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>321</v>
@@ -2979,19 +3007,19 @@
         <v>13</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I46" s="10" t="s">
         <v>323</v>
@@ -3011,19 +3039,19 @@
         <v>13</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>324</v>
@@ -3043,19 +3071,19 @@
         <v>13</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I48" s="10" t="s">
         <v>325</v>
@@ -3075,19 +3103,19 @@
         <v>13</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>326</v>
@@ -3107,19 +3135,19 @@
         <v>13</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I50" s="10" t="s">
         <v>327</v>
@@ -3139,19 +3167,19 @@
         <v>13</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I51" s="8" t="s">
         <v>328</v>
@@ -3168,22 +3196,22 @@
         <v>50</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I52" s="10" t="s">
         <v>329</v>
@@ -3203,19 +3231,19 @@
         <v>13</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="I53" s="8" t="s">
         <v>330</v>
@@ -3235,19 +3263,19 @@
         <v>13</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I54" s="10" t="s">
         <v>331</v>
@@ -3267,19 +3295,19 @@
         <v>13</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I55" s="8" t="s">
         <v>332</v>
@@ -3299,19 +3327,19 @@
         <v>13</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I56" s="10" t="s">
         <v>333</v>
@@ -3327,31 +3355,33 @@
         <f>ROW(B57) - ROW($B$2)</f>
         <v>55</v>
       </c>
-      <c r="C57" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="F57" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="G57" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="H57" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="I57" s="8" t="s">
+      <c r="C57" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D57" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E57" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="F57" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="G57" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="H57" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="I57" s="16" t="s">
         <v>322</v>
       </c>
-      <c r="J57" s="7">
+      <c r="J57" s="15">
         <v>9</v>
       </c>
-      <c r="K57" s="7"/>
+      <c r="K57" s="15" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
@@ -3360,25 +3390,25 @@
         <v>56</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H58" s="9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="I58" s="10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J58" s="9">
         <v>3</v>
@@ -3392,25 +3422,25 @@
         <v>57</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>290</v>
-      </c>
-      <c r="I59" s="8" t="s">
-        <v>340</v>
+        <v>291</v>
+      </c>
+      <c r="I59" s="10" t="s">
+        <v>339</v>
       </c>
       <c r="J59" s="7">
         <v>1</v>
@@ -3423,26 +3453,26 @@
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="C60" s="13" t="s">
-        <v>16</v>
+      <c r="C60" s="12" t="s">
+        <v>17</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J60" s="9">
         <v>1</v>
@@ -3456,25 +3486,25 @@
         <v>59</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>292</v>
-      </c>
-      <c r="I61" s="8" t="s">
-        <v>340</v>
+        <v>293</v>
+      </c>
+      <c r="I61" s="10" t="s">
+        <v>339</v>
       </c>
       <c r="J61" s="7">
         <v>1</v>
@@ -3488,25 +3518,25 @@
         <v>60</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J62" s="9">
         <v>1</v>
@@ -3520,25 +3550,25 @@
         <v>61</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="I63" s="8" t="s">
-        <v>340</v>
+        <v>295</v>
+      </c>
+      <c r="I63" s="10" t="s">
+        <v>339</v>
       </c>
       <c r="J63" s="7">
         <v>1</v>
@@ -3552,25 +3582,25 @@
         <v>62</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J64" s="9">
         <v>6</v>
@@ -3584,25 +3614,25 @@
         <v>63</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="I65" s="8" t="s">
-        <v>340</v>
+        <v>273</v>
+      </c>
+      <c r="I65" s="10" t="s">
+        <v>339</v>
       </c>
       <c r="J65" s="7">
         <v>1</v>
@@ -3616,25 +3646,25 @@
         <v>64</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I66" s="10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J66" s="9">
         <v>1</v>
@@ -3648,25 +3678,25 @@
         <v>65</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>296</v>
-      </c>
-      <c r="I67" s="8" t="s">
-        <v>340</v>
+        <v>297</v>
+      </c>
+      <c r="I67" s="10" t="s">
+        <v>339</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
@@ -3680,25 +3710,25 @@
         <v>66</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J68" s="9">
         <v>1</v>
@@ -3712,22 +3742,22 @@
         <v>67</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="I69" s="8" t="s">
         <v>334</v>
@@ -3744,22 +3774,22 @@
         <v>68</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="I70" s="10" t="s">
         <v>335</v>

</xml_diff>